<commit_message>
Rename synthetic project to Majmooeh Sepehr
</commit_message>
<xml_diff>
--- a/excel/HOMA-Analysis.xlsx
+++ b/excel/HOMA-Analysis.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="خلاصه" sheetId="1" r:id="R3bf894d268b64a70"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="پروژه‌ها" sheetId="2" r:id="Rd86c0fc2629740f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="خلاصه" sheetId="1" r:id="R640050b1e6da4c22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="پروژه‌ها" sheetId="2" r:id="R565c27c76dee4367"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1079,7 +1079,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="B16" s="3" t="str">
-        <x:v>پایانه مهر 1</x:v>
+        <x:v>مجموعه سپهر 1</x:v>
       </x:c>
       <x:c r="C16" s="3" t="str">
         <x:v>توسعه شهری</x:v>
@@ -1547,7 +1547,7 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="B28" s="3" t="str">
-        <x:v>پایانه مهر 2</x:v>
+        <x:v>مجموعه سپهر 2</x:v>
       </x:c>
       <x:c r="C28" s="3" t="str">
         <x:v>سازه و زیرساخت</x:v>
@@ -2015,7 +2015,7 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="B40" s="3" t="str">
-        <x:v>پایانه مهر 3</x:v>
+        <x:v>مجموعه سپهر 3</x:v>
       </x:c>
       <x:c r="C40" s="3" t="str">
         <x:v>ساخت صنعتی</x:v>
@@ -2483,7 +2483,7 @@
         <x:v>44</x:v>
       </x:c>
       <x:c r="B52" s="3" t="str">
-        <x:v>پایانه مهر 4</x:v>
+        <x:v>مجموعه سپهر 4</x:v>
       </x:c>
       <x:c r="C52" s="3" t="str">
         <x:v>بازآفرینی</x:v>
@@ -2951,7 +2951,7 @@
         <x:v>56</x:v>
       </x:c>
       <x:c r="B64" s="3" t="str">
-        <x:v>پایانه مهر 5</x:v>
+        <x:v>مجموعه سپهر 5</x:v>
       </x:c>
       <x:c r="C64" s="3" t="str">
         <x:v>تأسیسات و انرژی</x:v>

</xml_diff>